<commit_message>
fix: regenerate HTML+xlsx with rocm_ci_data.py present — InferenceMAX sheets now populated
</commit_message>
<xml_diff>
--- a/ROCm_CICD_Comprehensive.xlsx
+++ b/ROCm_CICD_Comprehensive.xlsx
@@ -20,9 +20,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Component CI Matrix'!$A$2:$V$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Framework Detail'!$A$1:$M$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Inference Runners'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Inference Runners'!$A$1:$E$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'InferenceMAX Workflows'!$A$2:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'InferenceMAX — AMD Benchmarks'!$A$2:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'InferenceMAX — AMD Benchmarks'!$A$2:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Runner Inventory'!$A$7:$K$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Wheel Artifact Publishing'!$A$1:$K$10</definedName>
   </definedNames>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2435" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2808" uniqueCount="817">
   <si>
     <t>Category</t>
   </si>
@@ -1832,6 +1832,285 @@
     <t>Pinned Docker Image</t>
   </si>
   <si>
+    <t>glm5-fp8-mi355x-atom</t>
+  </si>
+  <si>
+    <t>zai-org/GLM-5-FP8</t>
+  </si>
+  <si>
+    <t>glm5</t>
+  </si>
+  <si>
+    <t>mi355x</t>
+  </si>
+  <si>
+    <t>fp8</t>
+  </si>
+  <si>
+    <t>atom</t>
+  </si>
+  <si>
+    <t>rocm/atom-dev:nightly_202603291522</t>
+  </si>
+  <si>
+    <t>kimik2.5-fp4-mi355x-atom</t>
+  </si>
+  <si>
+    <t>amd/Kimi-K2.5-MXFP4</t>
+  </si>
+  <si>
+    <t>kimik2.5</t>
+  </si>
+  <si>
+    <t>fp4</t>
+  </si>
+  <si>
+    <t>rocm/atom-dev:nightly_202603251629</t>
+  </si>
+  <si>
+    <t>minimaxm2.5-fp8-mi355x-atom</t>
+  </si>
+  <si>
+    <t>MiniMaxAI/MiniMax-M2.5</t>
+  </si>
+  <si>
+    <t>minimaxm2.5</t>
+  </si>
+  <si>
+    <t>gptoss-fp4-mi355x-atom</t>
+  </si>
+  <si>
+    <t>openai/gpt-oss-120b</t>
+  </si>
+  <si>
+    <t>gptoss</t>
+  </si>
+  <si>
+    <t>dsr1-fp4-mi355x-atom-mtp</t>
+  </si>
+  <si>
+    <t>amd/DeepSeek-R1-0528-MXFP4-MTP-MoEFP4</t>
+  </si>
+  <si>
+    <t>dsr1</t>
+  </si>
+  <si>
+    <t>rocm/atom:rocm7.2.1-ubuntu24.04-pytorch2.9.1-atom0.1.2</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi355x-atom-mtp</t>
+  </si>
+  <si>
+    <t>deepseek-ai/DeepSeek-R1-0528</t>
+  </si>
+  <si>
+    <t>dsr1-fp4-mi355x-atom</t>
+  </si>
+  <si>
+    <t>amd/DeepSeek-R1-0528-MXFP4-Preview</t>
+  </si>
+  <si>
+    <t>rocm/atom:rocm7.1.1-ubuntu24.04-pytorch2.9-atom0.1.1-MI350x</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi355x-atom</t>
+  </si>
+  <si>
+    <t>dsv4-fp8-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>sgl-project/DeepSeek-V4-Pro-FP8</t>
+  </si>
+  <si>
+    <t>dsv4</t>
+  </si>
+  <si>
+    <t>sglang</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:rocm720-deepseek-v4-mi35x</t>
+  </si>
+  <si>
+    <t>dsv4-fp4-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>deepseek-ai/DeepSeek-V4-Pro</t>
+  </si>
+  <si>
+    <t>dsv4-fp4-mi355x-vllm</t>
+  </si>
+  <si>
+    <t>mi355x-p02-g57</t>
+  </si>
+  <si>
+    <t>vllm</t>
+  </si>
+  <si>
+    <t>rocm/pytorch-private:dsv4_dsv4_adapt_upstream_0430</t>
+  </si>
+  <si>
+    <t>dsr1-fp4-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>lmsysorg/sglang:v0.5.9-rocm700-mi35x</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi300x-sglang</t>
+  </si>
+  <si>
+    <t>mi300x</t>
+  </si>
+  <si>
+    <t>lmsysorg/sglang:v0.5.9-rocm700-mi30x</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi325x-sglang</t>
+  </si>
+  <si>
+    <t>mi325x</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>qwen3.5-bf16-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>Qwen/Qwen3.5-397B-A17B</t>
+  </si>
+  <si>
+    <t>qwen3.5</t>
+  </si>
+  <si>
+    <t>bf16</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:v0.5.8.post1-rocm720-mi35x-20260215</t>
+  </si>
+  <si>
+    <t>qwen3.5-bf16-mi355x-atom</t>
+  </si>
+  <si>
+    <t>rocm/atom:rocm7.2.1-ubuntu24.04-pytorch2.9.1-atom0.1.2-vllm0.17.0</t>
+  </si>
+  <si>
+    <t>qwen3.5-bf16-mi300x-sglang</t>
+  </si>
+  <si>
+    <t>lmsysorg/sglang:v0.5.9-rocm720-mi30x</t>
+  </si>
+  <si>
+    <t>qwen3.5-bf16-mi325x-sglang</t>
+  </si>
+  <si>
+    <t>qwen3.5-fp8-mi325x-sglang</t>
+  </si>
+  <si>
+    <t>Qwen/Qwen3.5-397B-A17B-FP8</t>
+  </si>
+  <si>
+    <t>qwen3.5-fp8-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:v0.5.8.post1-rocm720-mi35x-20260218</t>
+  </si>
+  <si>
+    <t>qwen3.5-fp8-mi355x-atom</t>
+  </si>
+  <si>
+    <t>qwen3.5-fp8-mi300x-sglang</t>
+  </si>
+  <si>
+    <t>glm5-fp8-mi355x-sglang</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:v0.5.8.post1-rocm720-mi35x-20260219</t>
+  </si>
+  <si>
+    <t>kimik2.5-int4-mi355x-vllm</t>
+  </si>
+  <si>
+    <t>moonshotai/Kimi-K2.5</t>
+  </si>
+  <si>
+    <t>mi355x_srok</t>
+  </si>
+  <si>
+    <t>int4</t>
+  </si>
+  <si>
+    <t>aigmkt/kimi-k25-dev</t>
+  </si>
+  <si>
+    <t>kimik2.5-int4-mi325x-vllm</t>
+  </si>
+  <si>
+    <t>vllm/vllm-openai-rocm:v0.18.0</t>
+  </si>
+  <si>
+    <t>kimik2.5-fp4-mi355x-vllm</t>
+  </si>
+  <si>
+    <t>mi355x-p02-g42</t>
+  </si>
+  <si>
+    <t>minimaxm2.5-fp8-mi355x-vllm</t>
+  </si>
+  <si>
+    <t>vllm/vllm-openai-rocm:v0.15.1</t>
+  </si>
+  <si>
+    <t>minimaxm2.5-fp8-mi300x-vllm</t>
+  </si>
+  <si>
+    <t>vllm/vllm-openai-rocm:v0.16.0</t>
+  </si>
+  <si>
+    <t>minimaxm2.5-fp8-mi325x-vllm</t>
+  </si>
+  <si>
+    <t>gptoss-fp4-mi300x-vllm</t>
+  </si>
+  <si>
+    <t>vllm/vllm-openai-rocm:v0.17.0</t>
+  </si>
+  <si>
+    <t>gptoss-fp4-mi325x-vllm</t>
+  </si>
+  <si>
+    <t>gptoss-fp4-mi355x-vllm</t>
+  </si>
+  <si>
+    <t>amd/gpt-oss-120b-w-mxfp4-a-fp8</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi355x-sglang-disagg</t>
+  </si>
+  <si>
+    <t>mi355x-disagg</t>
+  </si>
+  <si>
+    <t>sglang-disagg</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:sglang-0.5.9-rocm720-mi35x-mori-0227-2</t>
+  </si>
+  <si>
+    <t>dsr1-fp8-mi355x-sglang-disagg-mtp</t>
+  </si>
+  <si>
+    <t>dsr1-fp4-mi355x-sglang-disagg</t>
+  </si>
+  <si>
+    <t>amd/DeepSeek-R1-0528-MXFP4</t>
+  </si>
+  <si>
+    <t>rocm/sgl-dev:sglang-0.5.9-rocm720-mi35x-mori-0227-3</t>
+  </si>
+  <si>
+    <t>dsr1-fp4-mi355x-sglang-disagg-mtp</t>
+  </si>
+  <si>
     <t>Ecosystem</t>
   </si>
   <si>
@@ -1847,10 +2126,121 @@
     <t>Cluster Type</t>
   </si>
   <si>
+    <t>AMD</t>
+  </si>
+  <si>
+    <t>b200</t>
+  </si>
+  <si>
+    <t>b200-dgxc_1, b200-dgxc_2, b200-nb_0, b200-nb_1, b200-dgxc-slurm_0, b200-dgxc-slurm_1, b200-dgxc-slurm_2, b200-dgxc-slurm_3, b200-dgxc-slurm_4, b200-dgxc-slurm_5, b200-dgxc-slurm_6, b200-dgxc-slurm_7, b200-dgxc-slurm_8</t>
+  </si>
+  <si>
+    <t>SLURM</t>
+  </si>
+  <si>
+    <t>b200-multinode</t>
+  </si>
+  <si>
+    <t>b200-dgxc-slurm_6, b200-dgxc-slurm_7, b200-dgxc-slurm_8</t>
+  </si>
+  <si>
+    <t>b200-trt</t>
+  </si>
+  <si>
+    <t>b200-nb_0, b200-nb_1</t>
+  </si>
+  <si>
+    <t>Docker/Self-hosted</t>
+  </si>
+  <si>
+    <t>b300</t>
+  </si>
+  <si>
+    <t>b300-nv_0, b300-nv_1, b300-nv_2</t>
+  </si>
+  <si>
+    <t>gb200</t>
+  </si>
+  <si>
+    <t>gb200-nv_0, gb200-nv_1, gb200-nv_2</t>
+  </si>
+  <si>
+    <t>gb300</t>
+  </si>
+  <si>
+    <t>gb300-nv_0, gb300-nv_1, gb300-nv_2</t>
+  </si>
+  <si>
+    <t>h100</t>
+  </si>
+  <si>
+    <t>h100-cr_0, h100-cr_1, h100-cw_0, h100-cw_1, h100-dgxc-slurm_0, h100-dgxc-slurm_1, h100-dgxc-slurm_2, h100-dgxc-slurm_3, h100-dgxc-slurm_4, h100-dgxc-slurm_5, h100-dgxc-slurm_6, h100-dgxc-slurm_7, h100-dgxc-slurm_8, h100-dgxc-slurm_9, h100-dgxc-slurm_10, h100-dgxc-slurm_11</t>
+  </si>
+  <si>
+    <t>h100-multinode</t>
+  </si>
+  <si>
+    <t>h100-dgxc-slurm_9, h100-dgxc-slurm_10, h100-dgxc-slurm_11</t>
+  </si>
+  <si>
+    <t>h200</t>
+  </si>
+  <si>
+    <t>h200-cw_2, h200-cw_3, h200-nb_0, h200-nb_1, h200-dgxc-slurm_0, h200-dgxc-slurm_1, h200-dgxc-slurm_2, h200-dgxc-slurm_3, h200-dgxc-slurm_4, h200-dgxc-slurm_5, h200-dgxc-slurm_6, h200-dgxc-slurm_7, h200-dgxc-slurm_8, h200-dgxc-slurm_9, h200-dgxc-slurm_10, h200-dgxc-slurm_11, h200-dgxc-slurm_12, h200-dgxc-slurm_13</t>
+  </si>
+  <si>
+    <t>h200-multinode</t>
+  </si>
+  <si>
+    <t>h200-dgxc-slurm_11, h200-dgxc-slurm_12, h200-dgxc-slurm_13</t>
+  </si>
+  <si>
+    <t>mi300x-amd_0, mi300x-amd_1, mi300x-amd_2, mi300x-amd_3, mi300x-amd_4, mi300x-amds_0, mi300x-amds_1, mi300x-amds_2, mi300x-amds_3</t>
+  </si>
+  <si>
+    <t>mi325x-amd_0, mi325x-amd_1, mi325x-amd_2, mi325x-amd_3</t>
+  </si>
+  <si>
+    <t>mi355x-amds_0, mi355x-amds_1, mi355x-amds_2, mi355x-amds_3, mi355x-amds_4, mi355x-amds_5, mi355x-amds_6, mi355x-amds_7, mi355x-amds_8, mi355x-amd_p01_g06</t>
+  </si>
+  <si>
+    <t>mi355x-amds_0, mi355x-amds_1, mi355x-amds_2</t>
+  </si>
+  <si>
+    <t>mi355x-m15-17</t>
+  </si>
+  <si>
+    <t>mi355x-amd</t>
+  </si>
+  <si>
+    <t>mi355x-p02-g09</t>
+  </si>
+  <si>
+    <t>mi355x-amd_9</t>
+  </si>
+  <si>
+    <t>mi355x-p02-g17</t>
+  </si>
+  <si>
+    <t>mi355x-amd_17</t>
+  </si>
+  <si>
+    <t>mi355x-amd_42</t>
+  </si>
+  <si>
+    <t>mi355x-tw-sctrl</t>
+  </si>
+  <si>
+    <t>mi355x-amds</t>
+  </si>
+  <si>
     <t>Total AMD Inference Nodes</t>
   </si>
   <si>
-    <t>0 GPU pool types</t>
+    <t>b200: 13  •  b200-multinode: 3  •  b200-trt: 2  •  b300: 3  •  gb200: 3  •  gb300: 3  •  h100: 16  •  h100-multinode: 3  •  h200: 18  •  h200-multinode: 3  •  mi300x: 9  •  mi325x: 4  •  mi355x: 10  •  mi355x-disagg: 3  •  mi355x-m15-17: 1  •  mi355x-p02-g09: 1  •  mi355x-p02-g17: 1  •  mi355x-p02-g42: 1  •  mi355x-tw-sctrl: 1</t>
+  </si>
+  <si>
+    <t>19 GPU pool types</t>
   </si>
   <si>
     <t>InferenceMAX CI Workflows — ROCm/InferenceMAX_rocm (.github/workflows/)</t>
@@ -2248,7 +2638,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2412,6 +2802,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -2638,6 +3035,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF4E342E"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -2675,12 +3078,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5F5F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2748,7 +3145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2987,7 +3384,19 @@
     <xf numFmtId="0" fontId="1" fillId="33" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="35" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="33" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2996,52 +3405,52 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="36" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="37" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="37" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="38" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="38" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="39" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="40" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="41" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="41" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="42" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="42" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="43" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="44" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="45" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="46" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="46" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="47" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10790,14 +11199,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="2" width="39.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.7109375" customWidth="1"/>
-    <col min="4" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
@@ -10838,8 +11250,970 @@
         <v>560</v>
       </c>
     </row>
+    <row r="3" spans="1:8" ht="20" customHeight="1">
+      <c r="A3" s="20" t="s">
+        <v>561</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G3" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="20" customHeight="1">
+      <c r="A4" s="20" t="s">
+        <v>568</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>569</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G4" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="20" customHeight="1">
+      <c r="A5" s="20" t="s">
+        <v>573</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G5" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="20" customHeight="1">
+      <c r="A6" s="20" t="s">
+        <v>576</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>577</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G6" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="20" customHeight="1">
+      <c r="A7" s="20" t="s">
+        <v>579</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>580</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G7" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="20" customHeight="1">
+      <c r="A8" s="20" t="s">
+        <v>583</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G8" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="20" customHeight="1">
+      <c r="A9" s="20" t="s">
+        <v>585</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G9" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="20" customHeight="1">
+      <c r="A10" s="20" t="s">
+        <v>588</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G10" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="20" customHeight="1">
+      <c r="A11" s="20" t="s">
+        <v>589</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>590</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G11" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="20" customHeight="1">
+      <c r="A12" s="20" t="s">
+        <v>594</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G12" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="20" customHeight="1">
+      <c r="A13" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="B13" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>597</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G13" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="20" customHeight="1">
+      <c r="A14" s="20" t="s">
+        <v>600</v>
+      </c>
+      <c r="B14" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G14" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="20" customHeight="1">
+      <c r="A15" s="20" t="s">
+        <v>602</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F15" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G15" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="20" customHeight="1">
+      <c r="A16" s="20" t="s">
+        <v>605</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G16" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="20" customHeight="1">
+      <c r="A17" s="20" t="s">
+        <v>607</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G17" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="20" customHeight="1">
+      <c r="A18" s="20" t="s">
+        <v>608</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G18" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="20" customHeight="1">
+      <c r="A19" s="20" t="s">
+        <v>613</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G19" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="20" customHeight="1">
+      <c r="A20" s="20" t="s">
+        <v>615</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G20" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="20" customHeight="1">
+      <c r="A21" s="20" t="s">
+        <v>617</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>609</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>611</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G21" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H21" s="20" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="20" customHeight="1">
+      <c r="A22" s="20" t="s">
+        <v>618</v>
+      </c>
+      <c r="B22" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G22" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H22" s="20" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="20" customHeight="1">
+      <c r="A23" s="20" t="s">
+        <v>620</v>
+      </c>
+      <c r="B23" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G23" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="20" customHeight="1">
+      <c r="A24" s="20" t="s">
+        <v>622</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>566</v>
+      </c>
+      <c r="G24" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="20" customHeight="1">
+      <c r="A25" s="20" t="s">
+        <v>623</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>619</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>610</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G25" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="20" customHeight="1">
+      <c r="A26" s="20" t="s">
+        <v>624</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>562</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>563</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>592</v>
+      </c>
+      <c r="G26" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H26" s="20" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="20" customHeight="1">
+      <c r="A27" s="20" t="s">
+        <v>626</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>627</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>629</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G27" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H27" s="20" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="20" customHeight="1">
+      <c r="A28" s="20" t="s">
+        <v>631</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>627</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>629</v>
+      </c>
+      <c r="F28" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G28" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H28" s="20" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="20" customHeight="1">
+      <c r="A29" s="20" t="s">
+        <v>633</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>569</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>570</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>634</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G29" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H29" s="20" t="s">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="20" customHeight="1">
+      <c r="A30" s="20" t="s">
+        <v>635</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F30" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G30" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H30" s="20" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="20" customHeight="1">
+      <c r="A31" s="20" t="s">
+        <v>637</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G31" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="20" customHeight="1">
+      <c r="A32" s="20" t="s">
+        <v>639</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>574</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>575</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G32" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="20" customHeight="1">
+      <c r="A33" s="20" t="s">
+        <v>640</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>577</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>603</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F33" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G33" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H33" s="20" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="20" customHeight="1">
+      <c r="A34" s="20" t="s">
+        <v>642</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>577</v>
+      </c>
+      <c r="C34" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>606</v>
+      </c>
+      <c r="E34" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F34" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G34" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="20" customHeight="1">
+      <c r="A35" s="20" t="s">
+        <v>643</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>644</v>
+      </c>
+      <c r="C35" s="20" t="s">
+        <v>578</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>564</v>
+      </c>
+      <c r="E35" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F35" s="20" t="s">
+        <v>598</v>
+      </c>
+      <c r="G35" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="H35" s="20" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="20" customHeight="1">
+      <c r="A36" s="20" t="s">
+        <v>645</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="E36" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F36" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H36" s="20" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="20" customHeight="1">
+      <c r="A37" s="20" t="s">
+        <v>649</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>584</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>565</v>
+      </c>
+      <c r="F37" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H37" s="20" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="20" customHeight="1">
+      <c r="A38" s="20" t="s">
+        <v>650</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H38" s="20" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="20" customHeight="1">
+      <c r="A39" s="20" t="s">
+        <v>653</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>651</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>581</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>646</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>571</v>
+      </c>
+      <c r="F39" s="20" t="s">
+        <v>647</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H39" s="20" t="s">
+        <v>652</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H3"/>
+  <autoFilter ref="A2:H39"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -10849,7 +12223,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -10860,39 +12234,364 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="26" customHeight="1">
-      <c r="A1" s="80" t="s">
-        <v>561</v>
-      </c>
-      <c r="B1" s="80" t="s">
-        <v>562</v>
-      </c>
-      <c r="C1" s="80" t="s">
-        <v>563</v>
-      </c>
-      <c r="D1" s="80" t="s">
+      <c r="A1" s="81" t="s">
+        <v>654</v>
+      </c>
+      <c r="B1" s="81" t="s">
+        <v>655</v>
+      </c>
+      <c r="C1" s="81" t="s">
+        <v>656</v>
+      </c>
+      <c r="D1" s="81" t="s">
+        <v>657</v>
+      </c>
+      <c r="E1" s="81" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="20" customHeight="1">
+      <c r="A2" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B2" s="82" t="s">
+        <v>660</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>661</v>
+      </c>
+      <c r="D2" s="84">
+        <v>13</v>
+      </c>
+      <c r="E2" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="20" customHeight="1">
+      <c r="A3" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B3" s="82" t="s">
+        <v>663</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>664</v>
+      </c>
+      <c r="D3" s="84">
+        <v>3</v>
+      </c>
+      <c r="E3" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="20" customHeight="1">
+      <c r="A4" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B4" s="82" t="s">
+        <v>665</v>
+      </c>
+      <c r="C4" s="83" t="s">
+        <v>666</v>
+      </c>
+      <c r="D4" s="84">
+        <v>2</v>
+      </c>
+      <c r="E4" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="20" customHeight="1">
+      <c r="A5" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B5" s="82" t="s">
+        <v>668</v>
+      </c>
+      <c r="C5" s="83" t="s">
+        <v>669</v>
+      </c>
+      <c r="D5" s="84">
+        <v>3</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="20" customHeight="1">
+      <c r="A6" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B6" s="82" t="s">
+        <v>670</v>
+      </c>
+      <c r="C6" s="83" t="s">
+        <v>671</v>
+      </c>
+      <c r="D6" s="84">
+        <v>3</v>
+      </c>
+      <c r="E6" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="20" customHeight="1">
+      <c r="A7" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B7" s="82" t="s">
+        <v>672</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>673</v>
+      </c>
+      <c r="D7" s="84">
+        <v>3</v>
+      </c>
+      <c r="E7" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="20" customHeight="1">
+      <c r="A8" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B8" s="82" t="s">
+        <v>674</v>
+      </c>
+      <c r="C8" s="83" t="s">
+        <v>675</v>
+      </c>
+      <c r="D8" s="84">
+        <v>16</v>
+      </c>
+      <c r="E8" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="20" customHeight="1">
+      <c r="A9" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B9" s="82" t="s">
+        <v>676</v>
+      </c>
+      <c r="C9" s="83" t="s">
+        <v>677</v>
+      </c>
+      <c r="D9" s="84">
+        <v>3</v>
+      </c>
+      <c r="E9" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="20" customHeight="1">
+      <c r="A10" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B10" s="82" t="s">
+        <v>678</v>
+      </c>
+      <c r="C10" s="83" t="s">
+        <v>679</v>
+      </c>
+      <c r="D10" s="84">
+        <v>18</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="20" customHeight="1">
+      <c r="A11" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B11" s="82" t="s">
+        <v>680</v>
+      </c>
+      <c r="C11" s="83" t="s">
+        <v>681</v>
+      </c>
+      <c r="D11" s="84">
+        <v>3</v>
+      </c>
+      <c r="E11" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="20" customHeight="1">
+      <c r="A12" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B12" s="82" t="s">
+        <v>603</v>
+      </c>
+      <c r="C12" s="83" t="s">
+        <v>682</v>
+      </c>
+      <c r="D12" s="84">
+        <v>9</v>
+      </c>
+      <c r="E12" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="20" customHeight="1">
+      <c r="A13" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B13" s="82" t="s">
+        <v>606</v>
+      </c>
+      <c r="C13" s="83" t="s">
+        <v>683</v>
+      </c>
+      <c r="D13" s="84">
+        <v>4</v>
+      </c>
+      <c r="E13" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="20" customHeight="1">
+      <c r="A14" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B14" s="82" t="s">
         <v>564</v>
       </c>
-      <c r="E1" s="80" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="28" customHeight="1">
-      <c r="A2" s="81" t="s">
-        <v>566</v>
-      </c>
-      <c r="B2" s="81"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="81">
-        <v>0</v>
-      </c>
-      <c r="E2" s="81" t="s">
-        <v>567</v>
+      <c r="C14" s="83" t="s">
+        <v>684</v>
+      </c>
+      <c r="D14" s="84">
+        <v>10</v>
+      </c>
+      <c r="E14" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="20" customHeight="1">
+      <c r="A15" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B15" s="82" t="s">
+        <v>646</v>
+      </c>
+      <c r="C15" s="83" t="s">
+        <v>685</v>
+      </c>
+      <c r="D15" s="84">
+        <v>3</v>
+      </c>
+      <c r="E15" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="20" customHeight="1">
+      <c r="A16" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B16" s="82" t="s">
+        <v>686</v>
+      </c>
+      <c r="C16" s="83" t="s">
+        <v>687</v>
+      </c>
+      <c r="D16" s="84">
+        <v>1</v>
+      </c>
+      <c r="E16" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="20" customHeight="1">
+      <c r="A17" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B17" s="82" t="s">
+        <v>688</v>
+      </c>
+      <c r="C17" s="83" t="s">
+        <v>689</v>
+      </c>
+      <c r="D17" s="84">
+        <v>1</v>
+      </c>
+      <c r="E17" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="20" customHeight="1">
+      <c r="A18" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B18" s="82" t="s">
+        <v>690</v>
+      </c>
+      <c r="C18" s="83" t="s">
+        <v>691</v>
+      </c>
+      <c r="D18" s="84">
+        <v>1</v>
+      </c>
+      <c r="E18" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="20" customHeight="1">
+      <c r="A19" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B19" s="82" t="s">
+        <v>634</v>
+      </c>
+      <c r="C19" s="83" t="s">
+        <v>692</v>
+      </c>
+      <c r="D19" s="84">
+        <v>1</v>
+      </c>
+      <c r="E19" s="82" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="20" customHeight="1">
+      <c r="A20" s="82" t="s">
+        <v>659</v>
+      </c>
+      <c r="B20" s="82" t="s">
+        <v>693</v>
+      </c>
+      <c r="C20" s="83" t="s">
+        <v>694</v>
+      </c>
+      <c r="D20" s="84">
+        <v>1</v>
+      </c>
+      <c r="E20" s="82" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28" customHeight="1">
+      <c r="A21" s="85" t="s">
+        <v>695</v>
+      </c>
+      <c r="B21" s="85"/>
+      <c r="C21" s="86" t="s">
+        <v>696</v>
+      </c>
+      <c r="D21" s="85">
+        <v>98</v>
+      </c>
+      <c r="E21" s="85" t="s">
+        <v>697</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:E20"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10910,7 +12609,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
       <c r="A1" s="79" t="s">
-        <v>568</v>
+        <v>698</v>
       </c>
       <c r="B1" s="79"/>
       <c r="C1" s="79"/>
@@ -10922,314 +12621,314 @@
     </row>
     <row r="2" spans="1:8" ht="22" customHeight="1">
       <c r="A2" s="79" t="s">
-        <v>569</v>
+        <v>699</v>
       </c>
       <c r="B2" s="79" t="s">
-        <v>570</v>
+        <v>700</v>
       </c>
       <c r="C2" s="79" t="s">
-        <v>571</v>
+        <v>701</v>
       </c>
       <c r="D2" s="79" t="s">
-        <v>572</v>
+        <v>702</v>
       </c>
       <c r="E2" s="79" t="s">
-        <v>573</v>
+        <v>703</v>
       </c>
       <c r="F2" s="79" t="s">
-        <v>574</v>
+        <v>704</v>
       </c>
       <c r="G2" s="79" t="s">
-        <v>575</v>
+        <v>705</v>
       </c>
       <c r="H2" s="79" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="182" customHeight="1">
-      <c r="A3" s="83" t="s">
-        <v>576</v>
+      <c r="A3" s="87" t="s">
+        <v>706</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>577</v>
-      </c>
-      <c r="C3" s="84" t="s">
-        <v>578</v>
+        <v>707</v>
+      </c>
+      <c r="C3" s="88" t="s">
+        <v>708</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>579</v>
+        <v>709</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>580</v>
+        <v>710</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>581</v>
+        <v>711</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>582</v>
+        <v>712</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>583</v>
+        <v>713</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="20" customHeight="1">
-      <c r="A4" s="83" t="s">
-        <v>584</v>
+      <c r="A4" s="87" t="s">
+        <v>714</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>585</v>
-      </c>
-      <c r="C4" s="84" t="s">
-        <v>586</v>
+        <v>715</v>
+      </c>
+      <c r="C4" s="88" t="s">
+        <v>716</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>587</v>
+        <v>717</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>588</v>
+        <v>718</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>589</v>
+        <v>719</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>590</v>
+        <v>720</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="20" customHeight="1">
-      <c r="A5" s="83" t="s">
-        <v>591</v>
+      <c r="A5" s="87" t="s">
+        <v>721</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>592</v>
-      </c>
-      <c r="C5" s="84" t="s">
-        <v>586</v>
+        <v>722</v>
+      </c>
+      <c r="C5" s="88" t="s">
+        <v>716</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>587</v>
+        <v>717</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>593</v>
+        <v>723</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>589</v>
+        <v>719</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>594</v>
+        <v>724</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="84" customHeight="1">
-      <c r="A6" s="83" t="s">
-        <v>589</v>
+      <c r="A6" s="87" t="s">
+        <v>719</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>595</v>
-      </c>
-      <c r="C6" s="84" t="s">
-        <v>596</v>
+        <v>725</v>
+      </c>
+      <c r="C6" s="88" t="s">
+        <v>726</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>597</v>
+        <v>727</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>598</v>
+        <v>728</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>582</v>
+        <v>712</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>599</v>
+        <v>729</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="42" customHeight="1">
-      <c r="A7" s="83" t="s">
-        <v>600</v>
+      <c r="A7" s="87" t="s">
+        <v>730</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>601</v>
-      </c>
-      <c r="C7" s="84" t="s">
-        <v>602</v>
+        <v>731</v>
+      </c>
+      <c r="C7" s="88" t="s">
+        <v>732</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>603</v>
+        <v>733</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>604</v>
+        <v>734</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>605</v>
+        <v>735</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>606</v>
+        <v>736</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>607</v>
+        <v>737</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
-      <c r="A8" s="83" t="s">
-        <v>608</v>
+      <c r="A8" s="87" t="s">
+        <v>738</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>609</v>
-      </c>
-      <c r="C8" s="84" t="s">
-        <v>610</v>
+        <v>739</v>
+      </c>
+      <c r="C8" s="88" t="s">
+        <v>740</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>611</v>
+        <v>741</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>612</v>
+        <v>742</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>613</v>
+        <v>743</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>614</v>
+        <v>744</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="28" customHeight="1">
-      <c r="A9" s="83" t="s">
-        <v>615</v>
+      <c r="A9" s="87" t="s">
+        <v>745</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>616</v>
-      </c>
-      <c r="C9" s="84" t="s">
-        <v>617</v>
+        <v>746</v>
+      </c>
+      <c r="C9" s="88" t="s">
+        <v>747</v>
       </c>
       <c r="D9" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>618</v>
+        <v>748</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>619</v>
+        <v>749</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>620</v>
+        <v>750</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>621</v>
+        <v>751</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="20" customHeight="1">
-      <c r="A10" s="85" t="s">
-        <v>622</v>
-      </c>
-      <c r="B10" s="86" t="s">
-        <v>623</v>
-      </c>
-      <c r="C10" s="84" t="s">
-        <v>624</v>
-      </c>
-      <c r="D10" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="86" t="s">
-        <v>625</v>
-      </c>
-      <c r="F10" s="86" t="s">
-        <v>626</v>
-      </c>
-      <c r="G10" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" s="86" t="s">
-        <v>627</v>
+      <c r="A10" s="89" t="s">
+        <v>752</v>
+      </c>
+      <c r="B10" s="90" t="s">
+        <v>753</v>
+      </c>
+      <c r="C10" s="88" t="s">
+        <v>754</v>
+      </c>
+      <c r="D10" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="90" t="s">
+        <v>755</v>
+      </c>
+      <c r="F10" s="90" t="s">
+        <v>756</v>
+      </c>
+      <c r="G10" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="90" t="s">
+        <v>757</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="20" customHeight="1">
-      <c r="A11" s="85" t="s">
-        <v>628</v>
-      </c>
-      <c r="B11" s="86" t="s">
-        <v>629</v>
-      </c>
-      <c r="C11" s="84" t="s">
-        <v>624</v>
-      </c>
-      <c r="D11" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="86" t="s">
-        <v>630</v>
-      </c>
-      <c r="F11" s="86" t="s">
-        <v>631</v>
-      </c>
-      <c r="G11" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="H11" s="86" t="s">
-        <v>632</v>
+      <c r="A11" s="89" t="s">
+        <v>758</v>
+      </c>
+      <c r="B11" s="90" t="s">
+        <v>759</v>
+      </c>
+      <c r="C11" s="88" t="s">
+        <v>754</v>
+      </c>
+      <c r="D11" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="90" t="s">
+        <v>760</v>
+      </c>
+      <c r="F11" s="90" t="s">
+        <v>761</v>
+      </c>
+      <c r="G11" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="90" t="s">
+        <v>762</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="20" customHeight="1">
-      <c r="A12" s="85" t="s">
-        <v>633</v>
-      </c>
-      <c r="B12" s="86" t="s">
-        <v>634</v>
-      </c>
-      <c r="C12" s="84" t="s">
-        <v>635</v>
-      </c>
-      <c r="D12" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E12" s="86" t="s">
-        <v>636</v>
-      </c>
-      <c r="F12" s="86" t="s">
-        <v>637</v>
-      </c>
-      <c r="G12" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12" s="86" t="s">
-        <v>638</v>
+      <c r="A12" s="89" t="s">
+        <v>763</v>
+      </c>
+      <c r="B12" s="90" t="s">
+        <v>764</v>
+      </c>
+      <c r="C12" s="88" t="s">
+        <v>765</v>
+      </c>
+      <c r="D12" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="90" t="s">
+        <v>766</v>
+      </c>
+      <c r="F12" s="90" t="s">
+        <v>767</v>
+      </c>
+      <c r="G12" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="90" t="s">
+        <v>768</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="20" customHeight="1">
-      <c r="A13" s="85" t="s">
-        <v>639</v>
-      </c>
-      <c r="B13" s="86" t="s">
-        <v>640</v>
-      </c>
-      <c r="C13" s="84" t="s">
-        <v>641</v>
-      </c>
-      <c r="D13" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="E13" s="86" t="s">
-        <v>642</v>
-      </c>
-      <c r="F13" s="86" t="s">
-        <v>643</v>
-      </c>
-      <c r="G13" s="86" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" s="86" t="s">
-        <v>644</v>
+      <c r="A13" s="89" t="s">
+        <v>769</v>
+      </c>
+      <c r="B13" s="90" t="s">
+        <v>770</v>
+      </c>
+      <c r="C13" s="88" t="s">
+        <v>771</v>
+      </c>
+      <c r="D13" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="90" t="s">
+        <v>772</v>
+      </c>
+      <c r="F13" s="90" t="s">
+        <v>773</v>
+      </c>
+      <c r="G13" s="90" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" s="90" t="s">
+        <v>774</v>
       </c>
     </row>
   </sheetData>
@@ -11255,172 +12954,172 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
-      <c r="A1" s="87" t="s">
-        <v>645</v>
-      </c>
-      <c r="B1" s="87"/>
-      <c r="C1" s="87"/>
+      <c r="A1" s="91" t="s">
+        <v>775</v>
+      </c>
+      <c r="B1" s="91"/>
+      <c r="C1" s="91"/>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1">
-      <c r="A2" s="87" t="s">
-        <v>646</v>
-      </c>
-      <c r="B2" s="87" t="s">
-        <v>647</v>
-      </c>
-      <c r="C2" s="87" t="s">
-        <v>648</v>
+      <c r="A2" s="91" t="s">
+        <v>776</v>
+      </c>
+      <c r="B2" s="91" t="s">
+        <v>777</v>
+      </c>
+      <c r="C2" s="91" t="s">
+        <v>778</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
-      <c r="A3" s="88" t="s">
-        <v>649</v>
-      </c>
-      <c r="B3" s="89" t="s">
-        <v>650</v>
-      </c>
-      <c r="C3" s="90" t="s">
-        <v>651</v>
+      <c r="A3" s="92" t="s">
+        <v>779</v>
+      </c>
+      <c r="B3" s="93" t="s">
+        <v>780</v>
+      </c>
+      <c r="C3" s="94" t="s">
+        <v>781</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
-      <c r="A4" s="91" t="s">
-        <v>652</v>
-      </c>
-      <c r="B4" s="90" t="s">
-        <v>653</v>
-      </c>
-      <c r="C4" s="90" t="s">
-        <v>654</v>
+      <c r="A4" s="95" t="s">
+        <v>782</v>
+      </c>
+      <c r="B4" s="94" t="s">
+        <v>783</v>
+      </c>
+      <c r="C4" s="94" t="s">
+        <v>784</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
-      <c r="A5" s="91" t="s">
-        <v>655</v>
-      </c>
-      <c r="B5" s="90" t="s">
-        <v>656</v>
-      </c>
-      <c r="C5" s="90" t="s">
-        <v>657</v>
+      <c r="A5" s="95" t="s">
+        <v>785</v>
+      </c>
+      <c r="B5" s="94" t="s">
+        <v>786</v>
+      </c>
+      <c r="C5" s="94" t="s">
+        <v>787</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
-      <c r="A6" s="91" t="s">
-        <v>658</v>
-      </c>
-      <c r="B6" s="90" t="s">
-        <v>659</v>
-      </c>
-      <c r="C6" s="90" t="s">
-        <v>660</v>
+      <c r="A6" s="95" t="s">
+        <v>788</v>
+      </c>
+      <c r="B6" s="94" t="s">
+        <v>789</v>
+      </c>
+      <c r="C6" s="94" t="s">
+        <v>790</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
-      <c r="A7" s="91" t="s">
-        <v>661</v>
-      </c>
-      <c r="B7" s="90" t="s">
-        <v>662</v>
-      </c>
-      <c r="C7" s="90" t="s">
-        <v>663</v>
+      <c r="A7" s="95" t="s">
+        <v>791</v>
+      </c>
+      <c r="B7" s="94" t="s">
+        <v>792</v>
+      </c>
+      <c r="C7" s="94" t="s">
+        <v>793</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
-      <c r="A8" s="91" t="s">
-        <v>664</v>
-      </c>
-      <c r="B8" s="90" t="s">
-        <v>665</v>
-      </c>
-      <c r="C8" s="90" t="s">
-        <v>666</v>
+      <c r="A8" s="95" t="s">
+        <v>794</v>
+      </c>
+      <c r="B8" s="94" t="s">
+        <v>795</v>
+      </c>
+      <c r="C8" s="94" t="s">
+        <v>796</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
-      <c r="A9" s="91" t="s">
-        <v>667</v>
-      </c>
-      <c r="B9" s="90" t="s">
-        <v>668</v>
-      </c>
-      <c r="C9" s="90" t="s">
-        <v>669</v>
+      <c r="A9" s="95" t="s">
+        <v>797</v>
+      </c>
+      <c r="B9" s="94" t="s">
+        <v>798</v>
+      </c>
+      <c r="C9" s="94" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
-      <c r="A10" s="91" t="s">
-        <v>670</v>
-      </c>
-      <c r="B10" s="90" t="s">
-        <v>671</v>
-      </c>
-      <c r="C10" s="90" t="s">
-        <v>672</v>
+      <c r="A10" s="95" t="s">
+        <v>800</v>
+      </c>
+      <c r="B10" s="94" t="s">
+        <v>801</v>
+      </c>
+      <c r="C10" s="94" t="s">
+        <v>802</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
-      <c r="A11" s="92" t="s">
-        <v>673</v>
-      </c>
-      <c r="B11" s="93" t="s">
-        <v>674</v>
-      </c>
-      <c r="C11" s="90" t="s">
-        <v>675</v>
+      <c r="A11" s="96" t="s">
+        <v>803</v>
+      </c>
+      <c r="B11" s="97" t="s">
+        <v>804</v>
+      </c>
+      <c r="C11" s="94" t="s">
+        <v>805</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
-      <c r="A12" s="94" t="s">
-        <v>673</v>
-      </c>
-      <c r="B12" s="95" t="s">
-        <v>676</v>
-      </c>
-      <c r="C12" s="90" t="s">
-        <v>677</v>
+      <c r="A12" s="98" t="s">
+        <v>803</v>
+      </c>
+      <c r="B12" s="99" t="s">
+        <v>806</v>
+      </c>
+      <c r="C12" s="94" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
-      <c r="A13" s="96" t="s">
-        <v>678</v>
-      </c>
-      <c r="B13" s="97" t="s">
-        <v>679</v>
-      </c>
-      <c r="C13" s="90" t="s">
-        <v>680</v>
+      <c r="A13" s="100" t="s">
+        <v>808</v>
+      </c>
+      <c r="B13" s="101" t="s">
+        <v>809</v>
+      </c>
+      <c r="C13" s="94" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
-      <c r="A14" s="91" t="s">
-        <v>681</v>
-      </c>
-      <c r="B14" s="90" t="s">
-        <v>682</v>
-      </c>
-      <c r="C14" s="90" t="s">
-        <v>683</v>
+      <c r="A14" s="95" t="s">
+        <v>811</v>
+      </c>
+      <c r="B14" s="94" t="s">
+        <v>812</v>
+      </c>
+      <c r="C14" s="94" t="s">
+        <v>813</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
-      <c r="A15" s="91" t="s">
-        <v>684</v>
-      </c>
-      <c r="B15" s="90" t="s">
-        <v>685</v>
-      </c>
-      <c r="C15" s="98" t="s">
+      <c r="A15" s="95" t="s">
+        <v>814</v>
+      </c>
+      <c r="B15" s="94" t="s">
+        <v>815</v>
+      </c>
+      <c r="C15" s="102" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="30" customHeight="1">
-      <c r="A16" s="98" t="s">
-        <v>686</v>
-      </c>
-      <c r="B16" s="98"/>
-      <c r="C16" s="98"/>
+      <c r="A16" s="102" t="s">
+        <v>816</v>
+      </c>
+      <c r="B16" s="102"/>
+      <c r="C16" s="102"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
fix: split inference runners into AMD (mi*) and NVIDIA (h*/b*/gb*) ecosystems
runners.yaml contains both AMD and NVIDIA pools in one flat file.
create_snapshots.py and fetch_rocm_data.py were dumping all pools
into the 'amd' key, causing H100/H200/B200/GB200/GB300 to show
AMD badge in the Inference Runner Inventory section.

Fix: route pool_name.startswith('mi') -> amd, else -> nvidia.
generate_rocm_html.py now renders both AMD (red) and NVIDIA (green)
badge rows in the runner table.
</commit_message>
<xml_diff>
--- a/ROCm_CICD_Comprehensive.xlsx
+++ b/ROCm_CICD_Comprehensive.xlsx
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Component CI Matrix'!$A$2:$V$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Framework Detail'!$A$1:$M$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Inference Runners'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Inference Runners'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'InferenceMAX Workflows'!$A$2:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'InferenceMAX — AMD Benchmarks'!$A$2:$H$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Runner Inventory'!$A$7:$K$30</definedName>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2808" uniqueCount="817">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2768" uniqueCount="797">
   <si>
     <t>Category</t>
   </si>
@@ -2129,78 +2129,18 @@
     <t>AMD</t>
   </si>
   <si>
-    <t>b200</t>
-  </si>
-  <si>
-    <t>b200-dgxc_1, b200-dgxc_2, b200-nb_0, b200-nb_1, b200-dgxc-slurm_0, b200-dgxc-slurm_1, b200-dgxc-slurm_2, b200-dgxc-slurm_3, b200-dgxc-slurm_4, b200-dgxc-slurm_5, b200-dgxc-slurm_6, b200-dgxc-slurm_7, b200-dgxc-slurm_8</t>
+    <t>mi300x-amd_0, mi300x-amd_1, mi300x-amd_2, mi300x-amd_3, mi300x-amd_4, mi300x-amds_0, mi300x-amds_1, mi300x-amds_2, mi300x-amds_3</t>
   </si>
   <si>
     <t>SLURM</t>
   </si>
   <si>
-    <t>b200-multinode</t>
-  </si>
-  <si>
-    <t>b200-dgxc-slurm_6, b200-dgxc-slurm_7, b200-dgxc-slurm_8</t>
-  </si>
-  <si>
-    <t>b200-trt</t>
-  </si>
-  <si>
-    <t>b200-nb_0, b200-nb_1</t>
+    <t>mi325x-amd_0, mi325x-amd_1, mi325x-amd_2, mi325x-amd_3</t>
   </si>
   <si>
     <t>Docker/Self-hosted</t>
   </si>
   <si>
-    <t>b300</t>
-  </si>
-  <si>
-    <t>b300-nv_0, b300-nv_1, b300-nv_2</t>
-  </si>
-  <si>
-    <t>gb200</t>
-  </si>
-  <si>
-    <t>gb200-nv_0, gb200-nv_1, gb200-nv_2</t>
-  </si>
-  <si>
-    <t>gb300</t>
-  </si>
-  <si>
-    <t>gb300-nv_0, gb300-nv_1, gb300-nv_2</t>
-  </si>
-  <si>
-    <t>h100</t>
-  </si>
-  <si>
-    <t>h100-cr_0, h100-cr_1, h100-cw_0, h100-cw_1, h100-dgxc-slurm_0, h100-dgxc-slurm_1, h100-dgxc-slurm_2, h100-dgxc-slurm_3, h100-dgxc-slurm_4, h100-dgxc-slurm_5, h100-dgxc-slurm_6, h100-dgxc-slurm_7, h100-dgxc-slurm_8, h100-dgxc-slurm_9, h100-dgxc-slurm_10, h100-dgxc-slurm_11</t>
-  </si>
-  <si>
-    <t>h100-multinode</t>
-  </si>
-  <si>
-    <t>h100-dgxc-slurm_9, h100-dgxc-slurm_10, h100-dgxc-slurm_11</t>
-  </si>
-  <si>
-    <t>h200</t>
-  </si>
-  <si>
-    <t>h200-cw_2, h200-cw_3, h200-nb_0, h200-nb_1, h200-dgxc-slurm_0, h200-dgxc-slurm_1, h200-dgxc-slurm_2, h200-dgxc-slurm_3, h200-dgxc-slurm_4, h200-dgxc-slurm_5, h200-dgxc-slurm_6, h200-dgxc-slurm_7, h200-dgxc-slurm_8, h200-dgxc-slurm_9, h200-dgxc-slurm_10, h200-dgxc-slurm_11, h200-dgxc-slurm_12, h200-dgxc-slurm_13</t>
-  </si>
-  <si>
-    <t>h200-multinode</t>
-  </si>
-  <si>
-    <t>h200-dgxc-slurm_11, h200-dgxc-slurm_12, h200-dgxc-slurm_13</t>
-  </si>
-  <si>
-    <t>mi300x-amd_0, mi300x-amd_1, mi300x-amd_2, mi300x-amd_3, mi300x-amd_4, mi300x-amds_0, mi300x-amds_1, mi300x-amds_2, mi300x-amds_3</t>
-  </si>
-  <si>
-    <t>mi325x-amd_0, mi325x-amd_1, mi325x-amd_2, mi325x-amd_3</t>
-  </si>
-  <si>
     <t>mi355x-amds_0, mi355x-amds_1, mi355x-amds_2, mi355x-amds_3, mi355x-amds_4, mi355x-amds_5, mi355x-amds_6, mi355x-amds_7, mi355x-amds_8, mi355x-amd_p01_g06</t>
   </si>
   <si>
@@ -2237,10 +2177,10 @@
     <t>Total AMD Inference Nodes</t>
   </si>
   <si>
-    <t>b200: 13  •  b200-multinode: 3  •  b200-trt: 2  •  b300: 3  •  gb200: 3  •  gb300: 3  •  h100: 16  •  h100-multinode: 3  •  h200: 18  •  h200-multinode: 3  •  mi300x: 9  •  mi325x: 4  •  mi355x: 10  •  mi355x-disagg: 3  •  mi355x-m15-17: 1  •  mi355x-p02-g09: 1  •  mi355x-p02-g17: 1  •  mi355x-p02-g42: 1  •  mi355x-tw-sctrl: 1</t>
-  </si>
-  <si>
-    <t>19 GPU pool types</t>
+    <t>mi300x: 9  •  mi325x: 4  •  mi355x: 10  •  mi355x-disagg: 3  •  mi355x-m15-17: 1  •  mi355x-p02-g09: 1  •  mi355x-p02-g17: 1  •  mi355x-p02-g42: 1  •  mi355x-tw-sctrl: 1</t>
+  </si>
+  <si>
+    <t>9 GPU pool types</t>
   </si>
   <si>
     <t>InferenceMAX CI Workflows — ROCm/InferenceMAX_rocm (.github/workflows/)</t>
@@ -12223,7 +12163,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -12255,16 +12195,16 @@
         <v>659</v>
       </c>
       <c r="B2" s="82" t="s">
+        <v>603</v>
+      </c>
+      <c r="C2" s="83" t="s">
         <v>660</v>
       </c>
-      <c r="C2" s="83" t="s">
+      <c r="D2" s="84">
+        <v>9</v>
+      </c>
+      <c r="E2" s="82" t="s">
         <v>661</v>
-      </c>
-      <c r="D2" s="84">
-        <v>13</v>
-      </c>
-      <c r="E2" s="82" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20" customHeight="1">
@@ -12272,16 +12212,16 @@
         <v>659</v>
       </c>
       <c r="B3" s="82" t="s">
+        <v>606</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>662</v>
+      </c>
+      <c r="D3" s="84">
+        <v>4</v>
+      </c>
+      <c r="E3" s="82" t="s">
         <v>663</v>
-      </c>
-      <c r="C3" s="83" t="s">
-        <v>664</v>
-      </c>
-      <c r="D3" s="84">
-        <v>3</v>
-      </c>
-      <c r="E3" s="82" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20" customHeight="1">
@@ -12289,16 +12229,16 @@
         <v>659</v>
       </c>
       <c r="B4" s="82" t="s">
-        <v>665</v>
+        <v>564</v>
       </c>
       <c r="C4" s="83" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D4" s="84">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E4" s="82" t="s">
-        <v>667</v>
+        <v>661</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20" customHeight="1">
@@ -12306,16 +12246,16 @@
         <v>659</v>
       </c>
       <c r="B5" s="82" t="s">
-        <v>668</v>
+        <v>646</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="D5" s="84">
         <v>3</v>
       </c>
       <c r="E5" s="82" t="s">
-        <v>667</v>
+        <v>661</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="20" customHeight="1">
@@ -12323,16 +12263,16 @@
         <v>659</v>
       </c>
       <c r="B6" s="82" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="C6" s="83" t="s">
-        <v>671</v>
+        <v>667</v>
       </c>
       <c r="D6" s="84">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" s="82" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="20" customHeight="1">
@@ -12340,16 +12280,16 @@
         <v>659</v>
       </c>
       <c r="B7" s="82" t="s">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="C7" s="83" t="s">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="D7" s="84">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E7" s="82" t="s">
-        <v>667</v>
+        <v>663</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="20" customHeight="1">
@@ -12357,16 +12297,16 @@
         <v>659</v>
       </c>
       <c r="B8" s="82" t="s">
-        <v>674</v>
+        <v>670</v>
       </c>
       <c r="C8" s="83" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="D8" s="84">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="20" customHeight="1">
@@ -12374,16 +12314,16 @@
         <v>659</v>
       </c>
       <c r="B9" s="82" t="s">
-        <v>676</v>
+        <v>634</v>
       </c>
       <c r="C9" s="83" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="D9" s="84">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" s="82" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="20" customHeight="1">
@@ -12391,207 +12331,37 @@
         <v>659</v>
       </c>
       <c r="B10" s="82" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="C10" s="83" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="D10" s="84">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E10" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="20" customHeight="1">
-      <c r="A11" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B11" s="82" t="s">
-        <v>680</v>
-      </c>
-      <c r="C11" s="83" t="s">
-        <v>681</v>
-      </c>
-      <c r="D11" s="84">
-        <v>3</v>
-      </c>
-      <c r="E11" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="20" customHeight="1">
-      <c r="A12" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B12" s="82" t="s">
-        <v>603</v>
-      </c>
-      <c r="C12" s="83" t="s">
-        <v>682</v>
-      </c>
-      <c r="D12" s="84">
-        <v>9</v>
-      </c>
-      <c r="E12" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="20" customHeight="1">
-      <c r="A13" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B13" s="82" t="s">
-        <v>606</v>
-      </c>
-      <c r="C13" s="83" t="s">
-        <v>683</v>
-      </c>
-      <c r="D13" s="84">
-        <v>4</v>
-      </c>
-      <c r="E13" s="82" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="20" customHeight="1">
-      <c r="A14" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B14" s="82" t="s">
-        <v>564</v>
-      </c>
-      <c r="C14" s="83" t="s">
-        <v>684</v>
-      </c>
-      <c r="D14" s="84">
-        <v>10</v>
-      </c>
-      <c r="E14" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="20" customHeight="1">
-      <c r="A15" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B15" s="82" t="s">
-        <v>646</v>
-      </c>
-      <c r="C15" s="83" t="s">
-        <v>685</v>
-      </c>
-      <c r="D15" s="84">
-        <v>3</v>
-      </c>
-      <c r="E15" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="20" customHeight="1">
-      <c r="A16" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B16" s="82" t="s">
-        <v>686</v>
-      </c>
-      <c r="C16" s="83" t="s">
-        <v>687</v>
-      </c>
-      <c r="D16" s="84">
-        <v>1</v>
-      </c>
-      <c r="E16" s="82" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="20" customHeight="1">
-      <c r="A17" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B17" s="82" t="s">
-        <v>688</v>
-      </c>
-      <c r="C17" s="83" t="s">
-        <v>689</v>
-      </c>
-      <c r="D17" s="84">
-        <v>1</v>
-      </c>
-      <c r="E17" s="82" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="20" customHeight="1">
-      <c r="A18" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B18" s="82" t="s">
-        <v>690</v>
-      </c>
-      <c r="C18" s="83" t="s">
-        <v>691</v>
-      </c>
-      <c r="D18" s="84">
-        <v>1</v>
-      </c>
-      <c r="E18" s="82" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="20" customHeight="1">
-      <c r="A19" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B19" s="82" t="s">
-        <v>634</v>
-      </c>
-      <c r="C19" s="83" t="s">
-        <v>692</v>
-      </c>
-      <c r="D19" s="84">
-        <v>1</v>
-      </c>
-      <c r="E19" s="82" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="20" customHeight="1">
-      <c r="A20" s="82" t="s">
-        <v>659</v>
-      </c>
-      <c r="B20" s="82" t="s">
-        <v>693</v>
-      </c>
-      <c r="C20" s="83" t="s">
-        <v>694</v>
-      </c>
-      <c r="D20" s="84">
-        <v>1</v>
-      </c>
-      <c r="E20" s="82" t="s">
-        <v>662</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="28" customHeight="1">
-      <c r="A21" s="85" t="s">
-        <v>695</v>
-      </c>
-      <c r="B21" s="85"/>
-      <c r="C21" s="86" t="s">
-        <v>696</v>
-      </c>
-      <c r="D21" s="85">
-        <v>98</v>
-      </c>
-      <c r="E21" s="85" t="s">
-        <v>697</v>
+        <v>661</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="28" customHeight="1">
+      <c r="A11" s="85" t="s">
+        <v>675</v>
+      </c>
+      <c r="B11" s="85"/>
+      <c r="C11" s="86" t="s">
+        <v>676</v>
+      </c>
+      <c r="D11" s="85">
+        <v>31</v>
+      </c>
+      <c r="E11" s="85" t="s">
+        <v>677</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:E10"/>
   <mergeCells count="1">
-    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12609,7 +12379,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
       <c r="A1" s="79" t="s">
-        <v>698</v>
+        <v>678</v>
       </c>
       <c r="B1" s="79"/>
       <c r="C1" s="79"/>
@@ -12621,25 +12391,25 @@
     </row>
     <row r="2" spans="1:8" ht="22" customHeight="1">
       <c r="A2" s="79" t="s">
-        <v>699</v>
+        <v>679</v>
       </c>
       <c r="B2" s="79" t="s">
-        <v>700</v>
+        <v>680</v>
       </c>
       <c r="C2" s="79" t="s">
-        <v>701</v>
+        <v>681</v>
       </c>
       <c r="D2" s="79" t="s">
-        <v>702</v>
+        <v>682</v>
       </c>
       <c r="E2" s="79" t="s">
-        <v>703</v>
+        <v>683</v>
       </c>
       <c r="F2" s="79" t="s">
-        <v>704</v>
+        <v>684</v>
       </c>
       <c r="G2" s="79" t="s">
-        <v>705</v>
+        <v>685</v>
       </c>
       <c r="H2" s="79" t="s">
         <v>9</v>
@@ -12647,288 +12417,288 @@
     </row>
     <row r="3" spans="1:8" ht="182" customHeight="1">
       <c r="A3" s="87" t="s">
-        <v>706</v>
+        <v>686</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>707</v>
+        <v>687</v>
       </c>
       <c r="C3" s="88" t="s">
-        <v>708</v>
+        <v>688</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>709</v>
+        <v>689</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>710</v>
+        <v>690</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>711</v>
+        <v>691</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>712</v>
+        <v>692</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>713</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="20" customHeight="1">
       <c r="A4" s="87" t="s">
-        <v>714</v>
+        <v>694</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>715</v>
+        <v>695</v>
       </c>
       <c r="C4" s="88" t="s">
-        <v>716</v>
+        <v>696</v>
       </c>
       <c r="D4" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>717</v>
+        <v>697</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>718</v>
+        <v>698</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>719</v>
+        <v>699</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>720</v>
+        <v>700</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="20" customHeight="1">
       <c r="A5" s="87" t="s">
-        <v>721</v>
+        <v>701</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>722</v>
+        <v>702</v>
       </c>
       <c r="C5" s="88" t="s">
-        <v>716</v>
+        <v>696</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>717</v>
+        <v>697</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>723</v>
+        <v>703</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>719</v>
+        <v>699</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>724</v>
+        <v>704</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="84" customHeight="1">
       <c r="A6" s="87" t="s">
-        <v>719</v>
+        <v>699</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>725</v>
+        <v>705</v>
       </c>
       <c r="C6" s="88" t="s">
-        <v>726</v>
+        <v>706</v>
       </c>
       <c r="D6" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>727</v>
+        <v>707</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>728</v>
+        <v>708</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>712</v>
+        <v>692</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>729</v>
+        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="42" customHeight="1">
       <c r="A7" s="87" t="s">
-        <v>730</v>
+        <v>710</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>731</v>
+        <v>711</v>
       </c>
       <c r="C7" s="88" t="s">
-        <v>732</v>
+        <v>712</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>733</v>
+        <v>713</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>734</v>
+        <v>714</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>735</v>
+        <v>715</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>736</v>
+        <v>716</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>737</v>
+        <v>717</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
       <c r="A8" s="87" t="s">
-        <v>738</v>
+        <v>718</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>739</v>
+        <v>719</v>
       </c>
       <c r="C8" s="88" t="s">
-        <v>740</v>
+        <v>720</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>741</v>
+        <v>721</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>742</v>
+        <v>722</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>743</v>
+        <v>723</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>744</v>
+        <v>724</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="28" customHeight="1">
       <c r="A9" s="87" t="s">
-        <v>745</v>
+        <v>725</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>746</v>
+        <v>726</v>
       </c>
       <c r="C9" s="88" t="s">
-        <v>747</v>
+        <v>727</v>
       </c>
       <c r="D9" s="20" t="s">
         <v>22</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>748</v>
+        <v>728</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>749</v>
+        <v>729</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>750</v>
+        <v>730</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>751</v>
+        <v>731</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="20" customHeight="1">
       <c r="A10" s="89" t="s">
-        <v>752</v>
+        <v>732</v>
       </c>
       <c r="B10" s="90" t="s">
-        <v>753</v>
+        <v>733</v>
       </c>
       <c r="C10" s="88" t="s">
-        <v>754</v>
+        <v>734</v>
       </c>
       <c r="D10" s="90" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="90" t="s">
-        <v>755</v>
+        <v>735</v>
       </c>
       <c r="F10" s="90" t="s">
-        <v>756</v>
+        <v>736</v>
       </c>
       <c r="G10" s="90" t="s">
         <v>22</v>
       </c>
       <c r="H10" s="90" t="s">
-        <v>757</v>
+        <v>737</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="20" customHeight="1">
       <c r="A11" s="89" t="s">
-        <v>758</v>
+        <v>738</v>
       </c>
       <c r="B11" s="90" t="s">
-        <v>759</v>
+        <v>739</v>
       </c>
       <c r="C11" s="88" t="s">
-        <v>754</v>
+        <v>734</v>
       </c>
       <c r="D11" s="90" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="90" t="s">
-        <v>760</v>
+        <v>740</v>
       </c>
       <c r="F11" s="90" t="s">
-        <v>761</v>
+        <v>741</v>
       </c>
       <c r="G11" s="90" t="s">
         <v>22</v>
       </c>
       <c r="H11" s="90" t="s">
-        <v>762</v>
+        <v>742</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="20" customHeight="1">
       <c r="A12" s="89" t="s">
-        <v>763</v>
+        <v>743</v>
       </c>
       <c r="B12" s="90" t="s">
-        <v>764</v>
+        <v>744</v>
       </c>
       <c r="C12" s="88" t="s">
-        <v>765</v>
+        <v>745</v>
       </c>
       <c r="D12" s="90" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="90" t="s">
-        <v>766</v>
+        <v>746</v>
       </c>
       <c r="F12" s="90" t="s">
-        <v>767</v>
+        <v>747</v>
       </c>
       <c r="G12" s="90" t="s">
         <v>22</v>
       </c>
       <c r="H12" s="90" t="s">
-        <v>768</v>
+        <v>748</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="20" customHeight="1">
       <c r="A13" s="89" t="s">
-        <v>769</v>
+        <v>749</v>
       </c>
       <c r="B13" s="90" t="s">
-        <v>770</v>
+        <v>750</v>
       </c>
       <c r="C13" s="88" t="s">
-        <v>771</v>
+        <v>751</v>
       </c>
       <c r="D13" s="90" t="s">
         <v>22</v>
       </c>
       <c r="E13" s="90" t="s">
-        <v>772</v>
+        <v>752</v>
       </c>
       <c r="F13" s="90" t="s">
-        <v>773</v>
+        <v>753</v>
       </c>
       <c r="G13" s="90" t="s">
         <v>22</v>
       </c>
       <c r="H13" s="90" t="s">
-        <v>774</v>
+        <v>754</v>
       </c>
     </row>
   </sheetData>
@@ -12955,160 +12725,160 @@
   <sheetData>
     <row r="1" spans="1:3" ht="28" customHeight="1">
       <c r="A1" s="91" t="s">
-        <v>775</v>
+        <v>755</v>
       </c>
       <c r="B1" s="91"/>
       <c r="C1" s="91"/>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1">
       <c r="A2" s="91" t="s">
-        <v>776</v>
+        <v>756</v>
       </c>
       <c r="B2" s="91" t="s">
-        <v>777</v>
+        <v>757</v>
       </c>
       <c r="C2" s="91" t="s">
-        <v>778</v>
+        <v>758</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
       <c r="A3" s="92" t="s">
-        <v>779</v>
+        <v>759</v>
       </c>
       <c r="B3" s="93" t="s">
-        <v>780</v>
+        <v>760</v>
       </c>
       <c r="C3" s="94" t="s">
-        <v>781</v>
+        <v>761</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
       <c r="A4" s="95" t="s">
-        <v>782</v>
+        <v>762</v>
       </c>
       <c r="B4" s="94" t="s">
-        <v>783</v>
+        <v>763</v>
       </c>
       <c r="C4" s="94" t="s">
-        <v>784</v>
+        <v>764</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
       <c r="A5" s="95" t="s">
-        <v>785</v>
+        <v>765</v>
       </c>
       <c r="B5" s="94" t="s">
-        <v>786</v>
+        <v>766</v>
       </c>
       <c r="C5" s="94" t="s">
-        <v>787</v>
+        <v>767</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
       <c r="A6" s="95" t="s">
-        <v>788</v>
+        <v>768</v>
       </c>
       <c r="B6" s="94" t="s">
-        <v>789</v>
+        <v>769</v>
       </c>
       <c r="C6" s="94" t="s">
-        <v>790</v>
+        <v>770</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
       <c r="A7" s="95" t="s">
-        <v>791</v>
+        <v>771</v>
       </c>
       <c r="B7" s="94" t="s">
-        <v>792</v>
+        <v>772</v>
       </c>
       <c r="C7" s="94" t="s">
-        <v>793</v>
+        <v>773</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
       <c r="A8" s="95" t="s">
-        <v>794</v>
+        <v>774</v>
       </c>
       <c r="B8" s="94" t="s">
-        <v>795</v>
+        <v>775</v>
       </c>
       <c r="C8" s="94" t="s">
-        <v>796</v>
+        <v>776</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
       <c r="A9" s="95" t="s">
-        <v>797</v>
+        <v>777</v>
       </c>
       <c r="B9" s="94" t="s">
-        <v>798</v>
+        <v>778</v>
       </c>
       <c r="C9" s="94" t="s">
-        <v>799</v>
+        <v>779</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
       <c r="A10" s="95" t="s">
-        <v>800</v>
+        <v>780</v>
       </c>
       <c r="B10" s="94" t="s">
-        <v>801</v>
+        <v>781</v>
       </c>
       <c r="C10" s="94" t="s">
-        <v>802</v>
+        <v>782</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
       <c r="A11" s="96" t="s">
-        <v>803</v>
+        <v>783</v>
       </c>
       <c r="B11" s="97" t="s">
-        <v>804</v>
+        <v>784</v>
       </c>
       <c r="C11" s="94" t="s">
-        <v>805</v>
+        <v>785</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
       <c r="A12" s="98" t="s">
-        <v>803</v>
+        <v>783</v>
       </c>
       <c r="B12" s="99" t="s">
-        <v>806</v>
+        <v>786</v>
       </c>
       <c r="C12" s="94" t="s">
-        <v>807</v>
+        <v>787</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
       <c r="A13" s="100" t="s">
-        <v>808</v>
+        <v>788</v>
       </c>
       <c r="B13" s="101" t="s">
-        <v>809</v>
+        <v>789</v>
       </c>
       <c r="C13" s="94" t="s">
-        <v>810</v>
+        <v>790</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
       <c r="A14" s="95" t="s">
-        <v>811</v>
+        <v>791</v>
       </c>
       <c r="B14" s="94" t="s">
-        <v>812</v>
+        <v>792</v>
       </c>
       <c r="C14" s="94" t="s">
-        <v>813</v>
+        <v>793</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
       <c r="A15" s="95" t="s">
-        <v>814</v>
+        <v>794</v>
       </c>
       <c r="B15" s="94" t="s">
-        <v>815</v>
+        <v>795</v>
       </c>
       <c r="C15" s="102" t="s">
         <v>22</v>
@@ -13116,7 +12886,7 @@
     </row>
     <row r="16" spans="1:3" ht="30" customHeight="1">
       <c r="A16" s="102" t="s">
-        <v>816</v>
+        <v>796</v>
       </c>
       <c r="B16" s="102"/>
       <c r="C16" s="102"/>

</xml_diff>